<commit_message>
line classifier with accounts
</commit_message>
<xml_diff>
--- a/outputs/19_02_2026_COND�MINOS_DO_CONDOM�NIO_ARRECADA��O_MENSAL_-_FUNDO_DE_OBRA_-_M�S_ANT_000000_seens.xlsx
+++ b/outputs/19_02_2026_COND�MINOS_DO_CONDOM�NIO_ARRECADA��O_MENSAL_-_FUNDO_DE_OBRA_-_M�S_ANT_000000_seens.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A5:L79"/>
+  <dimension ref="A5:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="3" max="3"/>
@@ -499,104 +499,107 @@
       </c>
     </row>
     <row r="14">
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="n">
-        <v>7040</v>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>ARRECADAO MENSAL - FLUXO DE CAIXA DE MANUTENO - MS ANTERIOR</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>1760</v>
       </c>
     </row>
     <row r="15">
       <c r="C15" s="1" t="inlineStr">
         <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>8800</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="C16" s="1" t="inlineStr">
+        <is>
           <t>(+) RECEITAS DE COTAS</t>
         </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>CONSUMO INDIVIDUAL DE GUA - MS ANTERIOR</t>
-        </is>
-      </c>
-      <c r="L16" s="3" t="n">
-        <v>5222.89</v>
       </c>
     </row>
     <row r="17">
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>DESPESAS ORDINRIAS - MS ANTERIOR</t>
+          <t>CONSUMO INDIVIDUAL DE GUA - MS ANTERIOR</t>
         </is>
       </c>
       <c r="L17" s="3" t="n">
-        <v>11405.68</v>
+        <v>5222.89</v>
       </c>
     </row>
     <row r="18">
       <c r="C18" s="2" t="inlineStr">
         <is>
+          <t>DESPESAS ORDINRIAS - MS ANTERIOR</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>11405.68</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="2" t="inlineStr">
+        <is>
           <t>TAXA DE UTILIZAO DO SALAO DE FESTAS - APTO 64</t>
         </is>
       </c>
-      <c r="L18" s="3" t="n">
+      <c r="L19" s="3" t="n">
         <v>163.62</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="C19" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="n">
-        <v>16792.19</v>
       </c>
     </row>
     <row r="20">
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>(+) RECEITAS FINANCEIRAS</t>
-        </is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>16792.19</v>
       </c>
     </row>
     <row r="21">
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="n">
-        <v>0</v>
+          <t>(+) RECEITAS FINANCEIRAS</t>
+        </is>
       </c>
     </row>
     <row r="22">
-      <c r="C22" s="1" t="inlineStr">
-        <is>
-          <t>(-) DESPESAS DIVERSAS</t>
-        </is>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>RENDIMENTO PROVISIONADO: JUROS - IRRF DE APLICAO FINANCEIRA</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>938.98</v>
       </c>
     </row>
     <row r="23">
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>MATERIAL DE LIMPEZA PARA O CONDOMNIO - DIVERSOS - NF 26401</t>
+          <t>RENDIMENTO - JUROS DE POUPANA</t>
         </is>
       </c>
       <c r="L23" s="3" t="n">
-        <v>551.22</v>
+        <v>363.34</v>
       </c>
     </row>
     <row r="24">
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>MENSALIDADE SEGLINE - CERCA ELTRICA E SERVIOS POR EVENTO</t>
+          <t>RESGATE DESTINADO ENTRADA 50% COMPRA DA PORTA PRINCIPAL DO HALL</t>
         </is>
       </c>
       <c r="L24" s="3" t="n">
-        <v>224.63</v>
+        <v>7475</v>
       </c>
     </row>
     <row r="25">
@@ -606,34 +609,34 @@
         </is>
       </c>
       <c r="L25" s="4" t="n">
-        <v>775.85</v>
+        <v>8777.32</v>
       </c>
     </row>
     <row r="26">
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>(-) DESPESAS COM MANUTEN��O</t>
+          <t>(-) DESPESAS DIVERSAS</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>SERVIOS DE LIMPEZA CONDOMINIAL - EMPRESA TERCEIRIZADA</t>
+          <t>MATERIAL DE LIMPEZA PARA O CONDOMNIO - DIVERSOS - NF 26401</t>
         </is>
       </c>
       <c r="L27" s="3" t="n">
-        <v>2911.02</v>
+        <v>551.22</v>
       </c>
     </row>
     <row r="28">
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>MANUTENO MENSAL DO ELEVADOR - 9140483</t>
+          <t>MENSALIDADE SEGLINE - CERCA ELTRICA E SERVIOS POR EVENTO</t>
         </is>
       </c>
       <c r="L28" s="3" t="n">
-        <v>540.85</v>
+        <v>224.63</v>
       </c>
     </row>
     <row r="29">
@@ -643,34 +646,34 @@
         </is>
       </c>
       <c r="L29" s="4" t="n">
-        <v>3451.87</v>
+        <v>775.85</v>
       </c>
     </row>
     <row r="30">
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t>(-) GARANTIDORA</t>
+          <t>(-) DESPESAS COM MANUTEN��O</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>HONORRIOS DA GARANTIDORA FINANCEIRA (5%)</t>
+          <t>SERVIOS DE LIMPEZA CONDOMINIAL - EMPRESA TERCEIRIZADA</t>
         </is>
       </c>
       <c r="L31" s="3" t="n">
-        <v>1216.58</v>
+        <v>2911.02</v>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>TARIFA BANCRIA PARA EMISSO DE BOLETOS BANCRIOS - GARANTIDORA</t>
+          <t>MANUTENO MENSAL DO ELEVADOR - 9140483</t>
         </is>
       </c>
       <c r="L32" s="3" t="n">
-        <v>44</v>
+        <v>540.85</v>
       </c>
     </row>
     <row r="33">
@@ -680,439 +683,513 @@
         </is>
       </c>
       <c r="L33" s="4" t="n">
-        <v>1260.58</v>
+        <v>3451.87</v>
       </c>
     </row>
     <row r="34">
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t>(-) IMPOSTOS E TAXAS</t>
+          <t>(-) TARIFAS BANC�RIAS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>GUIA DE PREVIDNCIA SOCIAL AO INSS E OUTRAS ENTIDADES</t>
+          <t>COTA CAPITAL SOCIAL SICREDI - MENSAL</t>
         </is>
       </c>
       <c r="L35" s="3" t="n">
-        <v>846.92</v>
+        <v>16</v>
       </c>
     </row>
     <row r="36">
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>GUIA DE CSLL/COFINS/PIS</t>
+          <t>TARIFA PACOTE DE SERVIOS SICREDI PESSOA JURDICA</t>
         </is>
       </c>
       <c r="L36" s="3" t="n">
-        <v>26.38</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="37">
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>GUIA DE PREVIDNCIA SOCIAL AO INSS E OUTRAS ENTIDADES</t>
-        </is>
-      </c>
-      <c r="L37" s="3" t="n">
-        <v>408.69</v>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="n">
+        <v>31.6</v>
       </c>
     </row>
     <row r="38">
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="L38" s="4" t="n">
-        <v>1281.99</v>
+          <t>(-) GARANTIDORA</t>
+        </is>
       </c>
     </row>
     <row r="39">
-      <c r="C39" s="1" t="inlineStr">
-        <is>
-          <t>(-) DESPESAS DE CONSUMO</t>
-        </is>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>HONORRIOS DA GARANTIDORA FINANCEIRA (5%)</t>
+        </is>
+      </c>
+      <c r="L39" s="3" t="n">
+        <v>1216.58</v>
       </c>
     </row>
     <row r="40">
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>INTERNET PARA AS CMERAS DE SEGURANA - FATURA OI 2037048648</t>
+          <t>TARIFA BANCRIA PARA EMISSO DE BOLETOS BANCRIOS - GARANTIDORA</t>
         </is>
       </c>
       <c r="L40" s="3" t="n">
-        <v>122.33</v>
+        <v>44</v>
       </c>
     </row>
     <row r="41">
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>FORNECIMENTO DE ENERGIA P/ REAS COMUNS - 95231544</t>
-        </is>
-      </c>
-      <c r="L41" s="3" t="n">
-        <v>681.5599999999999</v>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="n">
+        <v>1260.58</v>
       </c>
     </row>
     <row r="42">
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>FORNEC. DE ENERGIA P/ ESCADA PRESSURIZADA - 95822321</t>
-        </is>
-      </c>
-      <c r="L42" s="3" t="n">
-        <v>90.52</v>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>(-) IMPOSTOS E TAXAS</t>
+        </is>
       </c>
     </row>
     <row r="43">
-      <c r="C43" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="L43" s="4" t="n">
-        <v>894.41</v>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>GUIA DE PREVIDNCIA SOCIAL AO INSS E OUTRAS ENTIDADES</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="n">
+        <v>846.92</v>
       </c>
     </row>
     <row r="44">
-      <c r="C44" s="1" t="inlineStr">
-        <is>
-          <t>(-) DESPESAS ADMINISTRATIVAS</t>
-        </is>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>GUIA DE CSLL/COFINS/PIS</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="n">
+        <v>26.38</v>
       </c>
     </row>
     <row r="45">
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>DISTRIBUIO DE ATA - 34 ASSEMBLEIA GERAL ORDINRIA</t>
+          <t>GUIA DE PREVIDNCIA SOCIAL AO INSS E OUTRAS ENTIDADES</t>
         </is>
       </c>
       <c r="L45" s="3" t="n">
-        <v>24.25</v>
+        <v>408.69</v>
       </c>
     </row>
     <row r="46">
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>REGISTRO DE ATA - 34 ASSEMBLEIA GERAL ORDINRIA</t>
-        </is>
-      </c>
-      <c r="L46" s="3" t="n">
-        <v>127.5</v>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L46" s="4" t="n">
+        <v>1281.99</v>
       </c>
     </row>
     <row r="47">
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>SERVIO DE GESTO ADMINISTRATIVA CONDOMINIAL - NF 47</t>
-        </is>
-      </c>
-      <c r="L47" s="3" t="n">
-        <v>548.5700000000001</v>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>(-) DESPESAS DE CONSUMO</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>SNDICO CARLOS EDUARDO NICOLEM HONORRIOS PELOS SERVIOS DE SNDICO</t>
+          <t>INTERNET PARA AS CMERAS DE SEGURANA - FATURA OI 2037048648</t>
         </is>
       </c>
       <c r="L48" s="3" t="n">
-        <v>2431.5</v>
+        <v>122.33</v>
       </c>
     </row>
     <row r="49">
-      <c r="C49" s="1" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>FORNECIMENTO DE ENERGIA P/ REAS COMUNS - 95231544</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="n">
+        <v>681.5599999999999</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>FORNEC. DE ENERGIA P/ ESCADA PRESSURIZADA - 95822321</t>
+        </is>
+      </c>
+      <c r="L50" s="3" t="n">
+        <v>90.52</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="C51" s="1" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="L49" s="4" t="n">
-        <v>3131.82</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="C50" s="1" t="inlineStr">
-        <is>
-          <t>(-) �GUA E ESGOTO - RATEIO EFETUADO CONFORME O CONSUMO DA UNIDADE</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>CONSUMO DE GUA E ESGOTO MS - 3253534</t>
-        </is>
-      </c>
-      <c r="L51" s="3" t="n">
-        <v>5122.2</v>
+      <c r="L51" s="4" t="n">
+        <v>894.41</v>
       </c>
     </row>
     <row r="52">
       <c r="C52" s="1" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="L52" s="4" t="n">
-        <v>5122.2</v>
+          <t>(-) DESPESAS ADMINISTRATIVAS</t>
+        </is>
       </c>
     </row>
     <row r="53">
-      <c r="C53" s="1" t="inlineStr">
-        <is>
-          <t>(-) MANUTEN��ES DIVERSAS - FUNDO DE MANUTEN��O</t>
-        </is>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>DISTRIBUIO DE ATA - 34 ASSEMBLEIA GERAL ORDINRIA</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="n">
+        <v>24.25</v>
       </c>
     </row>
     <row r="54">
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>PREST. DE SERVIOS DE MANUT. DO SISTEMA DE INCNDIO - NF 648 - PARCELA 02/02</t>
+          <t>REGISTRO DE ATA - 34 ASSEMBLEIA GERAL ORDINRIA</t>
         </is>
       </c>
       <c r="L54" s="3" t="n">
-        <v>361.09</v>
+        <v>127.5</v>
       </c>
     </row>
     <row r="55">
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>MATERIAL PARA A MANUTENO PAINEL ELETRONICO CISTERNAS</t>
+          <t>SERVIO DE GESTO ADMINISTRATIVA CONDOMINIAL - NF 47</t>
         </is>
       </c>
       <c r="L55" s="3" t="n">
-        <v>348</v>
+        <v>548.5700000000001</v>
       </c>
     </row>
     <row r="56">
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>SERVIO DE REINSTALAO ELETROIM E MOLA AREA PORTA HALL</t>
+          <t>SNDICO CARLOS EDUARDO NICOLEM HONORRIOS PELOS SERVIOS DE SNDICO</t>
         </is>
       </c>
       <c r="L56" s="3" t="n">
-        <v>220</v>
+        <v>2431.5</v>
       </c>
     </row>
     <row r="57">
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>SERVIO DE MANUTENO PAINEL ELETRONICO CISTERNAS + PLACA PORTO TRREO</t>
-        </is>
-      </c>
-      <c r="L57" s="3" t="n">
-        <v>480</v>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="n">
+        <v>3131.82</v>
       </c>
     </row>
     <row r="58">
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>ENTRADA 50% COMPRA PORTA PRINCIPAL DO HALL</t>
-        </is>
-      </c>
-      <c r="L58" s="3" t="n">
-        <v>7475</v>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t>(-) �GUA E ESGOTO - RATEIO EFETUADO CONFORME O CONSUMO DA UNIDADE</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>DESPESAS ORDINRIAS</t>
+          <t>CONSUMO DE GUA E ESGOTO MS - 3253534</t>
         </is>
       </c>
       <c r="L59" s="3" t="n">
-        <v>10828.12</v>
+        <v>5122.2</v>
       </c>
     </row>
     <row r="60">
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>DESPESAS GUA E ESGOTO</t>
-        </is>
-      </c>
-      <c r="L60" s="3" t="n">
+      <c r="C60" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L60" s="4" t="n">
         <v>5122.2</v>
       </c>
     </row>
     <row r="61">
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>DESPESAS FUNDO DE MANUTENO</t>
-        </is>
-      </c>
-      <c r="L61" s="3" t="n">
-        <v>8884.09</v>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>(-) MANUTEN��ES DIVERSAS - FUNDO DE MANUTEN��O</t>
+        </is>
       </c>
     </row>
     <row r="62">
-      <c r="C62" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="L62" s="4" t="n">
-        <v>33718.5</v>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>PREST. DE SERVIOS DE MANUT. DO SISTEMA DE INCNDIO - NF 648 - PARCELA 02/02</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="n">
+        <v>361.09</v>
       </c>
     </row>
     <row r="63">
-      <c r="C63" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL RECEITAS DO MÊS</t>
-        </is>
-      </c>
-      <c r="L63" s="4" t="n">
-        <v>58201.7</v>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>MATERIAL PARA A MANUTENO PAINEL ELETRONICO CISTERNAS</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="n">
+        <v>348</v>
       </c>
     </row>
     <row r="64">
-      <c r="C64" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL DESPESAS DO MÊS</t>
-        </is>
-      </c>
-      <c r="L64" s="4" t="n">
-        <v>74471.63</v>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>SERVIO DE REINSTALAO ELETROIM E MOLA AREA PORTA HALL</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="n">
+        <v>220</v>
       </c>
     </row>
     <row r="65">
-      <c r="C65" s="1" t="inlineStr">
-        <is>
-          <t>RESUMO DO MÊS</t>
-        </is>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>SERVIO DE MANUTENO PAINEL ELETRONICO CISTERNAS + PLACA PORTO TRREO</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="n">
+        <v>480</v>
       </c>
     </row>
     <row r="66">
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>RECEITAS</t>
+          <t>ENTRADA 50% COMPRA PORTA PRINCIPAL DO HALL</t>
         </is>
       </c>
       <c r="L66" s="3" t="n">
-        <v>58201.7</v>
+        <v>7475</v>
       </c>
     </row>
     <row r="67">
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>DESPESAS</t>
+          <t>DESPESAS ORDINRIAS</t>
         </is>
       </c>
       <c r="L67" s="3" t="n">
-        <v>74471.63</v>
+        <v>10828.12</v>
       </c>
     </row>
     <row r="68">
-      <c r="C68" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL (RECEITAS - DESPESAS)</t>
-        </is>
-      </c>
-      <c r="L68" s="4" t="n">
-        <v>-16269.93</v>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>DESPESAS GUA E ESGOTO</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="n">
+        <v>5122.2</v>
       </c>
     </row>
     <row r="69">
-      <c r="C69" s="1" t="inlineStr">
-        <is>
-          <t>RESUMO DAS CONTAS - POSIÇÃO CONSOLIDADA DA CONTA PESSOA JURÍDICA - SICREDI</t>
-        </is>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>DESPESAS FUNDO DE MANUTENO</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="n">
+        <v>8884.09</v>
       </c>
     </row>
     <row r="70">
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>CONTAS CORRENTES</t>
-        </is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L70" s="4" t="n">
+        <v>33718.5</v>
       </c>
     </row>
     <row r="71">
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>SALDO ANTERIOR</t>
-        </is>
-      </c>
-      <c r="L71" s="3" t="n">
-        <v>0</v>
+      <c r="C71" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL RECEITAS DO MÊS</t>
+        </is>
+      </c>
+      <c r="L71" s="4" t="n">
+        <v>68739.02</v>
       </c>
     </row>
     <row r="72">
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>ENTRADAS</t>
-        </is>
-      </c>
-      <c r="L72" s="3" t="n">
-        <v>119726.96</v>
+      <c r="C72" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL DESPESAS DO MÊS</t>
+        </is>
+      </c>
+      <c r="L72" s="4" t="n">
+        <v>74503.23</v>
       </c>
     </row>
     <row r="73">
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>SAÍDAS</t>
-        </is>
-      </c>
-      <c r="L73" s="3" t="n">
-        <v>0</v>
+      <c r="C73" s="1" t="inlineStr">
+        <is>
+          <t>RESUMO DO MÊS</t>
+        </is>
       </c>
     </row>
     <row r="74">
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>SALDO ATUAL</t>
+          <t>RECEITAS</t>
         </is>
       </c>
       <c r="L74" s="3" t="n">
-        <v>95767.57000000001</v>
+        <v>68739.02</v>
       </c>
     </row>
     <row r="75">
-      <c r="C75" s="1" t="inlineStr">
-        <is>
-          <t>POUPAN�A</t>
-        </is>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>DESPESAS</t>
+        </is>
+      </c>
+      <c r="L75" s="3" t="n">
+        <v>74503.23</v>
       </c>
     </row>
     <row r="76">
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>SALDO ANTERIOR</t>
-        </is>
-      </c>
-      <c r="L76" s="3" t="n">
-        <v>0</v>
+      <c r="C76" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL (RECEITAS - DESPESAS)</t>
+        </is>
+      </c>
+      <c r="L76" s="4" t="n">
+        <v>-5764.21</v>
       </c>
     </row>
     <row r="77">
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>ENTRADAS</t>
-        </is>
-      </c>
-      <c r="L77" s="3" t="n">
-        <v>79631.71000000001</v>
+      <c r="C77" s="1" t="inlineStr">
+        <is>
+          <t>RESUMO DAS CONTAS - POSIÇÃO CONSOLIDADA DA CONTA PESSOA JURÍDICA - SICREDI</t>
+        </is>
       </c>
     </row>
     <row r="78">
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>SAÍDAS</t>
-        </is>
-      </c>
-      <c r="L78" s="3" t="n">
-        <v>0</v>
+      <c r="C78" s="1" t="inlineStr">
+        <is>
+          <t>CONTAS CORRENTES</t>
+        </is>
       </c>
     </row>
     <row r="79">
       <c r="C79" s="2" t="inlineStr">
         <is>
+          <t>SALDO ANTERIOR</t>
+        </is>
+      </c>
+      <c r="L79" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>ENTRADAS</t>
+        </is>
+      </c>
+      <c r="L80" s="3" t="n">
+        <v>119726.96</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>SAÍDAS</t>
+        </is>
+      </c>
+      <c r="L81" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="C82" s="2" t="inlineStr">
+        <is>
           <t>SALDO ATUAL</t>
         </is>
       </c>
-      <c r="L79" s="3" t="n">
+      <c r="L82" s="3" t="n">
+        <v>95767.57000000001</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="C83" s="1" t="inlineStr">
+        <is>
+          <t>POUPAN�A</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>SALDO ANTERIOR</t>
+        </is>
+      </c>
+      <c r="L84" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>ENTRADAS</t>
+        </is>
+      </c>
+      <c r="L85" s="3" t="n">
+        <v>79631.71000000001</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>SAÍDAS</t>
+        </is>
+      </c>
+      <c r="L86" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>SALDO ATUAL</t>
+        </is>
+      </c>
+      <c r="L87" s="3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
check for belle chateau
</commit_message>
<xml_diff>
--- a/outputs/19_02_2026_COND�MINOS_DO_CONDOM�NIO_ARRECADA��O_MENSAL_-_FUNDO_DE_OBRA_-_M�S_ANT_000000_seens.xlsx
+++ b/outputs/19_02_2026_COND�MINOS_DO_CONDOM�NIO_ARRECADA��O_MENSAL_-_FUNDO_DE_OBRA_-_M�S_ANT_000000_seens.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A5:L87"/>
+  <dimension ref="A5:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="3" max="3"/>
@@ -996,201 +996,218 @@
       </c>
     </row>
     <row r="67">
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>DESPESAS ORDINRIAS</t>
-        </is>
-      </c>
-      <c r="L67" s="3" t="n">
-        <v>10828.12</v>
+      <c r="C67" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L67" s="4" t="n">
+        <v>8884.09</v>
       </c>
     </row>
     <row r="68">
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>DESPESAS GUA E ESGOTO</t>
-        </is>
-      </c>
-      <c r="L68" s="3" t="n">
-        <v>5122.2</v>
+      <c r="C68" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL RECEITAS DO MÊS</t>
+        </is>
+      </c>
+      <c r="L68" s="4" t="n">
+        <v>34369.51</v>
       </c>
     </row>
     <row r="69">
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>DESPESAS FUNDO DE MANUTENO</t>
-        </is>
-      </c>
-      <c r="L69" s="3" t="n">
-        <v>8884.09</v>
+      <c r="C69" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL DESPESAS DO MÊS</t>
+        </is>
+      </c>
+      <c r="L69" s="4" t="n">
+        <v>24834.41</v>
       </c>
     </row>
     <row r="70">
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="L70" s="4" t="n">
-        <v>33718.5</v>
+          <t>RESUMO DO MÊS</t>
+        </is>
       </c>
     </row>
     <row r="71">
-      <c r="C71" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL RECEITAS DO MÊS</t>
-        </is>
-      </c>
-      <c r="L71" s="4" t="n">
-        <v>68739.02</v>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>RECEITAS</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="n">
+        <v>34369.51</v>
       </c>
     </row>
     <row r="72">
-      <c r="C72" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL DESPESAS DO MÊS</t>
-        </is>
-      </c>
-      <c r="L72" s="4" t="n">
-        <v>74503.23</v>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>DESPESAS</t>
+        </is>
+      </c>
+      <c r="L72" s="3" t="n">
+        <v>24834.41</v>
       </c>
     </row>
     <row r="73">
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>RESUMO DO MÊS</t>
-        </is>
+          <t>TOTAL (RECEITAS - DESPESAS)</t>
+        </is>
+      </c>
+      <c r="L73" s="4" t="n">
+        <v>9535.1</v>
       </c>
     </row>
     <row r="74">
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>RECEITAS</t>
-        </is>
-      </c>
-      <c r="L74" s="3" t="n">
-        <v>68739.02</v>
+      <c r="C74" s="1" t="inlineStr">
+        <is>
+          <t>RESUMO DAS CONTAS - POSIÇÃO CONSOLIDADA DA CONTA PESSOA JURÍDICA - SICREDI</t>
+        </is>
       </c>
     </row>
     <row r="75">
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>DESPESAS</t>
-        </is>
-      </c>
-      <c r="L75" s="3" t="n">
-        <v>74503.23</v>
+      <c r="C75" s="1" t="inlineStr">
+        <is>
+          <t>FUNDO DE OBRA</t>
+        </is>
       </c>
     </row>
     <row r="76">
-      <c r="C76" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL (RECEITAS - DESPESAS)</t>
-        </is>
-      </c>
-      <c r="L76" s="4" t="n">
-        <v>-5764.21</v>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>SALDO ANTERIOR</t>
+        </is>
+      </c>
+      <c r="L76" s="3" t="n">
+        <v>89988.59</v>
       </c>
     </row>
     <row r="77">
-      <c r="C77" s="1" t="inlineStr">
-        <is>
-          <t>RESUMO DAS CONTAS - POSIÇÃO CONSOLIDADA DA CONTA PESSOA JURÍDICA - SICREDI</t>
-        </is>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>ENTRADAS</t>
+        </is>
+      </c>
+      <c r="L77" s="3" t="n">
+        <v>5778.98</v>
       </c>
     </row>
     <row r="78">
-      <c r="C78" s="1" t="inlineStr">
-        <is>
-          <t>CONTAS CORRENTES</t>
-        </is>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>SAÍDAS</t>
+        </is>
+      </c>
+      <c r="L78" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="79">
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>SALDO ANTERIOR</t>
+          <t>SALDO ATUAL</t>
         </is>
       </c>
       <c r="L79" s="3" t="n">
-        <v>0</v>
+        <v>95767.57000000001</v>
       </c>
     </row>
     <row r="80">
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>ENTRADAS</t>
-        </is>
-      </c>
-      <c r="L80" s="3" t="n">
-        <v>119726.96</v>
+      <c r="C80" s="1" t="inlineStr">
+        <is>
+          <t>FUNDO DE RESERVA DE POUPANÇA PERMANENTE</t>
+        </is>
       </c>
     </row>
     <row r="81">
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>SAÍDAS</t>
+          <t>SALDO ANTERIOR</t>
         </is>
       </c>
       <c r="L81" s="3" t="n">
-        <v>0</v>
+        <v>69593.37</v>
       </c>
     </row>
     <row r="82">
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>SALDO ATUAL</t>
+          <t>ENTRADAS</t>
         </is>
       </c>
       <c r="L82" s="3" t="n">
-        <v>95767.57000000001</v>
+        <v>2563.34</v>
       </c>
     </row>
     <row r="83">
-      <c r="C83" s="1" t="inlineStr">
-        <is>
-          <t>POUPAN�A</t>
-        </is>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>SAÍDAS</t>
+        </is>
+      </c>
+      <c r="L83" s="3" t="n">
+        <v>7475</v>
       </c>
     </row>
     <row r="84">
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>SALDO ANTERIOR</t>
+          <t>SALDO ATUAL</t>
         </is>
       </c>
       <c r="L84" s="3" t="n">
-        <v>0</v>
+        <v>64681.71</v>
       </c>
     </row>
     <row r="85">
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>ENTRADAS</t>
-        </is>
-      </c>
-      <c r="L85" s="3" t="n">
-        <v>79631.71000000001</v>
+      <c r="C85" s="1" t="inlineStr">
+        <is>
+          <t>CONTA CORRENTE - FLUXO DE CAIXA DE MANUTENÇÃO</t>
+        </is>
       </c>
     </row>
     <row r="86">
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>SAÍDAS</t>
+          <t>SALDO ANTERIOR</t>
         </is>
       </c>
       <c r="L86" s="3" t="n">
-        <v>0</v>
+        <v>5407.2</v>
       </c>
     </row>
     <row r="87">
       <c r="C87" s="2" t="inlineStr">
         <is>
+          <t>ENTRADAS</t>
+        </is>
+      </c>
+      <c r="L87" s="3" t="n">
+        <v>26027.19</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>SAÍDAS</t>
+        </is>
+      </c>
+      <c r="L88" s="3" t="n">
+        <v>24834.41</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="C89" s="2" t="inlineStr">
+        <is>
           <t>SALDO ATUAL</t>
         </is>
       </c>
-      <c r="L87" s="3" t="n">
-        <v>0</v>
+      <c r="L89" s="3" t="n">
+        <v>6599.98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>